<commit_message>
Repair analytics, dashboard and release pipeline per audit backlog
Work through the 59-item master fix backlog (audit/MASTER_FIX_BACKLOG.md):
- Analytics: coverage-aware marts, null costs and matched windows, web
  grain/contact activity, duration eligibility, tie-preserving calibration,
  weekly-presence attribution, identity normalization, diagnostics.
- Frontend: typed sorting/units, chart labels and data alternatives,
  presenter sync/routes/timer, keyboard and modal fixes, responsive
  controls, print rules, traceable CSV exports, shared branding/fonts.
- Release: strict readiness and schema checks, public-field privacy gates,
  CI/Pages and Docker/Render gates, regenerated data and built assets.
- Tests: 41 Python and 16 frontend regressions; audit receipts in audit/.

Open dependencies (F16, F18, F40, F41, F54, F55-F59) are recorded in
audit/FIX_VERIFICATION.md.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/analysis/advanced_analytics.xlsx
+++ b/outputs/analysis/advanced_analytics.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="301" uniqueCount="176">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="378" uniqueCount="218">
   <si>
     <t>auc</t>
   </si>
@@ -67,22 +67,76 @@
     <t>active_scored_rows</t>
   </si>
   <si>
+    <t>canonical_resolved_rows</t>
+  </si>
+  <si>
+    <t>canonical_active_rows</t>
+  </si>
+  <si>
     <t>validation</t>
   </si>
   <si>
     <t>feature_policy</t>
   </si>
   <si>
+    <t>model_limitation</t>
+  </si>
+  <si>
+    <t>validation_cutoff</t>
+  </si>
+  <si>
+    <t>observation_end</t>
+  </si>
+  <si>
+    <t>outcome_horizon_days</t>
+  </si>
+  <si>
+    <t>mature_creation_rows</t>
+  </si>
+  <si>
+    <t>horizon_resolved_rows</t>
+  </si>
+  <si>
+    <t>ambiguous_outcome_rows</t>
+  </si>
+  <si>
+    <t>train_latest_resolution</t>
+  </si>
+  <si>
+    <t>test_earliest_creation</t>
+  </si>
+  <si>
+    <t>test_latest_horizon_end</t>
+  </si>
+  <si>
     <t>calibration_mean_abs_gap</t>
   </si>
   <si>
     <t>calibration_max_abs_gap</t>
   </si>
   <si>
-    <t>time-based 80/20 holdout; preprocessing fit on train only</t>
-  </si>
-  <si>
-    <t>opportunity-time fields only; present-day account snapshot fields excluded</t>
+    <t>as-of cutoff; train horizon and recorded resolution &lt;= cutoff; test creation &gt; cutoff and 180-day horizon &lt;= latest recorded event; preprocessing fit on train only</t>
+  </si>
+  <si>
+    <t>creation year/quarter only; mutable latest amount, channel, segment and account fields excluded</t>
+  </si>
+  <si>
+    <t>Exploratory calendar baseline conditional on first recorded resolution within 180 days; incomplete event coverage and resolved-only selection prevent unconditional active-deal win forecasting.</t>
+  </si>
+  <si>
+    <t>2024-01-22 00:00:00+00:00</t>
+  </si>
+  <si>
+    <t>2024-12-24 19:33:40+00:00</t>
+  </si>
+  <si>
+    <t>2023-12-20 16:41:38+00:00</t>
+  </si>
+  <si>
+    <t>2024-01-23 00:00:00+00:00</t>
+  </si>
+  <si>
+    <t>2024-12-24 00:00:00+00:00</t>
   </si>
   <si>
     <t>score_band</t>
@@ -91,28 +145,31 @@
     <t>n</t>
   </si>
   <si>
+    <t>wins</t>
+  </si>
+  <si>
     <t>predicted_win_rate</t>
   </si>
   <si>
     <t>observed_win_rate</t>
   </si>
   <si>
+    <t>score_min</t>
+  </si>
+  <si>
+    <t>score_max</t>
+  </si>
+  <si>
+    <t>observed_ci_low</t>
+  </si>
+  <si>
+    <t>observed_ci_high</t>
+  </si>
+  <si>
     <t>abs_gap</t>
   </si>
   <si>
-    <t>Test quintile 1</t>
-  </si>
-  <si>
-    <t>Test quintile 2</t>
-  </si>
-  <si>
-    <t>Test quintile 3</t>
-  </si>
-  <si>
-    <t>Test quintile 4</t>
-  </si>
-  <si>
-    <t>Test quintile 5</t>
+    <t>(25%,50%]</t>
   </si>
   <si>
     <t>feature</t>
@@ -121,319 +178,388 @@
     <t>importance</t>
   </si>
   <si>
+    <t>create_year</t>
+  </si>
+  <si>
+    <t>create_quarter</t>
+  </si>
+  <si>
+    <t>_opportunity_id</t>
+  </si>
+  <si>
+    <t>_account_name</t>
+  </si>
+  <si>
+    <t>_current_stage</t>
+  </si>
+  <si>
+    <t>_amount</t>
+  </si>
+  <si>
     <t>channel_category</t>
   </si>
   <si>
-    <t>_amount</t>
-  </si>
-  <si>
-    <t>create_year</t>
-  </si>
-  <si>
     <t>segment__c</t>
   </si>
   <si>
-    <t>create_quarter</t>
-  </si>
-  <si>
-    <t>_opportunity_id</t>
-  </si>
-  <si>
-    <t>_account_name</t>
-  </si>
-  <si>
-    <t>_current_stage</t>
-  </si>
-  <si>
     <t>win_probability</t>
   </si>
   <si>
+    <t>score_interpretation</t>
+  </si>
+  <si>
     <t>amount_quality</t>
   </si>
   <si>
+    <t>0064P00000rhpggQAA</t>
+  </si>
+  <si>
+    <t>0064P00000s9LVYQA2</t>
+  </si>
+  <si>
+    <t>0064P00000sXKP7QAO</t>
+  </si>
+  <si>
+    <t>0064P00000sa86lQAA</t>
+  </si>
+  <si>
+    <t>0064P00000rWItSQAW</t>
+  </si>
+  <si>
+    <t>0064P00000rZkTKQA0</t>
+  </si>
+  <si>
     <t>0064P00000uwKrzQAE</t>
   </si>
   <si>
+    <t>0064P00000uduBpQAI</t>
+  </si>
+  <si>
+    <t>0064P00000uxUTwQAM</t>
+  </si>
+  <si>
+    <t>0064P00000uwwS5QAI</t>
+  </si>
+  <si>
+    <t>0064P00000uw5dOQAQ</t>
+  </si>
+  <si>
     <t>0064P00000tSTnQQAW</t>
   </si>
   <si>
-    <t>006UW000007kI4MYAU</t>
-  </si>
-  <si>
-    <t>006UW00000JVboVYAT</t>
-  </si>
-  <si>
-    <t>006UW00000FpC3JYAV</t>
-  </si>
-  <si>
-    <t>006UW00000JGV89YAH</t>
-  </si>
-  <si>
-    <t>006UW00000JVyGIYA1</t>
-  </si>
-  <si>
-    <t>006UW00000I6MczYAF</t>
-  </si>
-  <si>
-    <t>006UW00000IzjdlYAB</t>
-  </si>
-  <si>
-    <t>006UW00000I4TKQYA3</t>
-  </si>
-  <si>
-    <t>006UW00000HVmjJYAT</t>
-  </si>
-  <si>
-    <t>006UW00000ByG0VYAV</t>
-  </si>
-  <si>
-    <t>006UW00000EMwLRYA1</t>
-  </si>
-  <si>
-    <t>006UW000001Pq4YYAS</t>
-  </si>
-  <si>
-    <t>006UW000001PtVQYA0</t>
-  </si>
-  <si>
-    <t>006UW00000Fati6YAB</t>
-  </si>
-  <si>
-    <t>006UW00000G3cAnYAJ</t>
-  </si>
-  <si>
-    <t>006UW00000Gz1M9YAJ</t>
-  </si>
-  <si>
-    <t>006UW00000HNj2fYAD</t>
-  </si>
-  <si>
-    <t>006UW00000HNjfNYAT</t>
+    <t>0064P00000td7ynQAA</t>
+  </si>
+  <si>
+    <t>0064P00000txWzWQAU</t>
+  </si>
+  <si>
+    <t>0064P00000xZgjSQAS</t>
+  </si>
+  <si>
+    <t>0064P00000xXFzZQAW</t>
+  </si>
+  <si>
+    <t>0064P00000xYlzEQAS</t>
+  </si>
+  <si>
+    <t>0064P00000xZ1T2QAK</t>
+  </si>
+  <si>
+    <t>0064P00000xYroXQAS</t>
+  </si>
+  <si>
+    <t>0064P00000xXGICQA4</t>
+  </si>
+  <si>
+    <t>Sigga</t>
+  </si>
+  <si>
+    <t>Vology</t>
+  </si>
+  <si>
+    <t>Nozomi Networks Inc</t>
+  </si>
+  <si>
+    <t>Argano</t>
+  </si>
+  <si>
+    <t>PRO</t>
+  </si>
+  <si>
+    <t>Y-Charts</t>
   </si>
   <si>
     <t>Enboarder</t>
   </si>
   <si>
+    <t>Crowdanalytix</t>
+  </si>
+  <si>
+    <t>Evolve Blue</t>
+  </si>
+  <si>
+    <t>LogicGate</t>
+  </si>
+  <si>
+    <t>SimScale GmbH</t>
+  </si>
+  <si>
     <t>IntelliShift</t>
   </si>
   <si>
-    <t>ConnectWise, Inc.</t>
-  </si>
-  <si>
-    <t>Elsevier</t>
-  </si>
-  <si>
-    <t>Randstad</t>
-  </si>
-  <si>
-    <t>Smart Communications</t>
-  </si>
-  <si>
-    <t>Novata</t>
-  </si>
-  <si>
-    <t>Seismic</t>
-  </si>
-  <si>
-    <t>S&amp;P Global</t>
-  </si>
-  <si>
-    <t>Gibraltar Industries</t>
-  </si>
-  <si>
-    <t>OFX</t>
-  </si>
-  <si>
-    <t>SAP</t>
-  </si>
-  <si>
-    <t>Rackspace</t>
-  </si>
-  <si>
-    <t>SEI</t>
+    <t>Intelity</t>
+  </si>
+  <si>
+    <t>RHR International</t>
+  </si>
+  <si>
+    <t>Capstorm, LLC</t>
+  </si>
+  <si>
+    <t>Tellius Inc</t>
+  </si>
+  <si>
+    <t>Drift</t>
+  </si>
+  <si>
+    <t>LS Direct Marketing</t>
+  </si>
+  <si>
+    <t>Okta Inc</t>
   </si>
   <si>
     <t>2: Discovery Call</t>
   </si>
   <si>
-    <t>6: Negotiate</t>
-  </si>
-  <si>
-    <t>5: Solution Scoping</t>
-  </si>
-  <si>
-    <t>6.5: Started Needs Paperwork</t>
-  </si>
-  <si>
-    <t>4: Qualified Opportunity</t>
+    <t>1: Marketing High Scoring Lead</t>
   </si>
   <si>
     <t>referral</t>
   </si>
   <si>
+    <t>6sense_channel</t>
+  </si>
+  <si>
+    <t>other</t>
+  </si>
+  <si>
     <t>existing_client</t>
   </si>
   <si>
+    <t>6sense_event</t>
+  </si>
+  <si>
     <t>Commercial</t>
   </si>
   <si>
     <t>Enterprise</t>
   </si>
   <si>
+    <t>Exploratory calendar baseline; conditional 180-day recorded-resolution outcome, not an operating win probability</t>
+  </si>
+  <si>
+    <t>positive amount</t>
+  </si>
+  <si>
+    <t>zero/missing amount</t>
+  </si>
+  <si>
+    <t>coverage_tier</t>
+  </si>
+  <si>
+    <t>accounts</t>
+  </si>
+  <si>
+    <t>with_opp</t>
+  </si>
+  <si>
+    <t>pct_of_total</t>
+  </si>
+  <si>
+    <t>opp_rate</t>
+  </si>
+  <si>
+    <t>opp_rate_ci_low</t>
+  </si>
+  <si>
+    <t>opp_rate_ci_high</t>
+  </si>
+  <si>
+    <t>interpretation</t>
+  </si>
+  <si>
+    <t>population_label</t>
+  </si>
+  <si>
+    <t>metric_definition</t>
+  </si>
+  <si>
+    <t>outcome_period</t>
+  </si>
+  <si>
+    <t>reach_period</t>
+  </si>
+  <si>
+    <t>email_reach_start</t>
+  </si>
+  <si>
+    <t>email_reach_end</t>
+  </si>
+  <si>
+    <t>6sense_reach_start</t>
+  </si>
+  <si>
+    <t>6sense_reach_end</t>
+  </si>
+  <si>
+    <t>historical_opportunity_prevalence</t>
+  </si>
+  <si>
+    <t>6sense Only</t>
+  </si>
+  <si>
+    <t>Both Channels</t>
+  </si>
+  <si>
+    <t>Email Only</t>
+  </si>
+  <si>
+    <t>Not Reached</t>
+  </si>
+  <si>
+    <t>Historical opportunity prevalence in all CRM history associated with reach in supplied activity windows; many opportunities predate reach. Not post-exposure conversion or a test baseline.</t>
+  </si>
+  <si>
+    <t>CRM account domains</t>
+  </si>
+  <si>
+    <t>Domains with any canonical historical opportunity / CRM account domains in coverage group</t>
+  </si>
+  <si>
+    <t>All supplied CRM history</t>
+  </si>
+  <si>
+    <t>Supplied email and 6sense activity windows</t>
+  </si>
+  <si>
+    <t>2024-01-01T15:41:43.395000+00:00</t>
+  </si>
+  <si>
+    <t>2024-12-23T19:52:58.312000+00:00</t>
+  </si>
+  <si>
+    <t>2024-02-01T00:00:00+00:00</t>
+  </si>
+  <si>
+    <t>2024-09-03T00:00:00+00:00</t>
+  </si>
+  <si>
+    <t>mean_days</t>
+  </si>
+  <si>
+    <t>median_days</t>
+  </si>
+  <si>
+    <t>deal_count</t>
+  </si>
+  <si>
+    <t>p25</t>
+  </si>
+  <si>
+    <t>p75</t>
+  </si>
+  <si>
+    <t>canonical_wins</t>
+  </si>
+  <si>
+    <t>included_share</t>
+  </si>
+  <si>
+    <t>eligibility_note</t>
+  </si>
+  <si>
+    <t>other_marketing</t>
+  </si>
+  <si>
+    <t>web_inbound</t>
+  </si>
+  <si>
+    <t>webinar</t>
+  </si>
+  <si>
+    <t>event</t>
+  </si>
+  <si>
+    <t>Includes same-day wins; excludes negative, missing and &gt;730-day intervals. See exclusions by channel/motion.</t>
+  </si>
+  <si>
+    <t>sequence_2ch</t>
+  </si>
+  <si>
+    <t>deals</t>
+  </si>
+  <si>
+    <t>pipeline</t>
+  </si>
+  <si>
+    <t>email_mqa</t>
+  </si>
+  <si>
+    <t>email_mqa -&gt; 6sense_display</t>
+  </si>
+  <si>
+    <t>6sense_display</t>
+  </si>
+  <si>
+    <t>6sense_display -&gt; email_mqa</t>
+  </si>
+  <si>
+    <t>is_6qa</t>
+  </si>
+  <si>
+    <t>won</t>
+  </si>
+  <si>
+    <t>won_pipeline</t>
+  </si>
+  <si>
+    <t>avg_deal</t>
+  </si>
+  <si>
+    <t>win_rate</t>
+  </si>
+  <si>
+    <t>accountprofilefit6sense__c</t>
+  </si>
+  <si>
+    <t>resolved_deals</t>
+  </si>
+  <si>
+    <t>positive_median_deal</t>
+  </si>
+  <si>
+    <t>total_deals</t>
+  </si>
+  <si>
+    <t>active_deals</t>
+  </si>
+  <si>
+    <t>adjusted_win_rate</t>
+  </si>
+  <si>
+    <t>win_rate_ci_low</t>
+  </si>
+  <si>
+    <t>win_rate_ci_high</t>
+  </si>
+  <si>
+    <t>evidence_tier</t>
+  </si>
+  <si>
+    <t>priority_score</t>
+  </si>
+  <si>
     <t>Mid</t>
-  </si>
-  <si>
-    <t>positive amount</t>
-  </si>
-  <si>
-    <t>zero/missing amount</t>
-  </si>
-  <si>
-    <t>coverage_tier</t>
-  </si>
-  <si>
-    <t>accounts</t>
-  </si>
-  <si>
-    <t>with_opp</t>
-  </si>
-  <si>
-    <t>pct_of_total</t>
-  </si>
-  <si>
-    <t>opp_rate</t>
-  </si>
-  <si>
-    <t>opp_rate_ci_low</t>
-  </si>
-  <si>
-    <t>opp_rate_ci_high</t>
-  </si>
-  <si>
-    <t>interpretation</t>
-  </si>
-  <si>
-    <t>population_label</t>
-  </si>
-  <si>
-    <t>6sense Only</t>
-  </si>
-  <si>
-    <t>Both Channels</t>
-  </si>
-  <si>
-    <t>Email Only</t>
-  </si>
-  <si>
-    <t>Not Reached</t>
-  </si>
-  <si>
-    <t>Observed association; coverage groups were not randomized.</t>
-  </si>
-  <si>
-    <t>CRM account domains</t>
-  </si>
-  <si>
-    <t>mean_days</t>
-  </si>
-  <si>
-    <t>median_days</t>
-  </si>
-  <si>
-    <t>deal_count</t>
-  </si>
-  <si>
-    <t>p25</t>
-  </si>
-  <si>
-    <t>p75</t>
-  </si>
-  <si>
-    <t>other_marketing</t>
-  </si>
-  <si>
-    <t>other</t>
-  </si>
-  <si>
-    <t>web_inbound</t>
-  </si>
-  <si>
-    <t>6sense_event</t>
-  </si>
-  <si>
-    <t>webinar</t>
-  </si>
-  <si>
-    <t>event</t>
-  </si>
-  <si>
-    <t>6sense_channel</t>
-  </si>
-  <si>
-    <t>6sense_display</t>
-  </si>
-  <si>
-    <t>sequence_2ch</t>
-  </si>
-  <si>
-    <t>deals</t>
-  </si>
-  <si>
-    <t>pipeline</t>
-  </si>
-  <si>
-    <t>email_mqa</t>
-  </si>
-  <si>
-    <t>email_mqa -&gt; 6sense_display</t>
-  </si>
-  <si>
-    <t>6sense_display -&gt; email_mqa</t>
-  </si>
-  <si>
-    <t>is_6qa</t>
-  </si>
-  <si>
-    <t>won</t>
-  </si>
-  <si>
-    <t>won_pipeline</t>
-  </si>
-  <si>
-    <t>avg_deal</t>
-  </si>
-  <si>
-    <t>win_rate</t>
-  </si>
-  <si>
-    <t>accountprofilefit6sense__c</t>
-  </si>
-  <si>
-    <t>resolved_deals</t>
-  </si>
-  <si>
-    <t>positive_median_deal</t>
-  </si>
-  <si>
-    <t>total_deals</t>
-  </si>
-  <si>
-    <t>active_deals</t>
-  </si>
-  <si>
-    <t>adjusted_win_rate</t>
-  </si>
-  <si>
-    <t>win_rate_ci_low</t>
-  </si>
-  <si>
-    <t>win_rate_ci_high</t>
-  </si>
-  <si>
-    <t>evidence_tier</t>
-  </si>
-  <si>
-    <t>priority_score</t>
   </si>
   <si>
     <t>Strong</t>
@@ -882,10 +1008,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R2"/>
+  <dimension ref="A1:AD2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:18">
+    <row r="1" spans="1:30">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -940,61 +1066,133 @@
       <c r="R1" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="2" spans="1:18">
+      <c r="S1" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" t="s">
+        <v>19</v>
+      </c>
+      <c r="U1" t="s">
+        <v>20</v>
+      </c>
+      <c r="V1" t="s">
+        <v>21</v>
+      </c>
+      <c r="W1" t="s">
+        <v>22</v>
+      </c>
+      <c r="X1" t="s">
+        <v>23</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Z1" t="s">
+        <v>25</v>
+      </c>
+      <c r="AA1" t="s">
+        <v>26</v>
+      </c>
+      <c r="AB1" t="s">
+        <v>27</v>
+      </c>
+      <c r="AC1" t="s">
+        <v>28</v>
+      </c>
+      <c r="AD1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2" spans="1:30">
       <c r="A2">
-        <v>0.7116434616434616</v>
+        <v>0.5163636363636364</v>
       </c>
       <c r="B2">
-        <v>0.7609841827768014</v>
+        <v>0.7674418604651163</v>
       </c>
       <c r="C2">
-        <v>0.6101694915254238</v>
+        <v>0</v>
       </c>
       <c r="D2">
-        <v>0.4444444444444444</v>
+        <v>0</v>
       </c>
       <c r="E2">
-        <v>0.1815009512802137</v>
+        <v>0.2170327636033189</v>
       </c>
       <c r="F2">
-        <v>361</v>
+        <v>330</v>
       </c>
       <c r="G2">
-        <v>46</v>
+        <v>0</v>
       </c>
       <c r="H2">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="I2">
-        <v>72</v>
+        <v>0</v>
       </c>
       <c r="J2">
-        <v>2272</v>
+        <v>1144</v>
       </c>
       <c r="K2">
-        <v>569</v>
+        <v>430</v>
       </c>
       <c r="L2">
-        <v>0.4009683098591549</v>
+        <v>0.5725524475524476</v>
       </c>
       <c r="M2">
-        <v>0.2847100175746924</v>
+        <v>0.2325581395348837</v>
       </c>
       <c r="N2">
-        <v>447</v>
-      </c>
-      <c r="O2" t="s">
-        <v>18</v>
-      </c>
-      <c r="P2" t="s">
-        <v>19</v>
-      </c>
-      <c r="Q2">
-        <v>0.06537146047494578</v>
-      </c>
-      <c r="R2">
-        <v>0.1394232562769266</v>
+        <v>411</v>
+      </c>
+      <c r="O2">
+        <v>2834</v>
+      </c>
+      <c r="P2">
+        <v>411</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>30</v>
+      </c>
+      <c r="R2" t="s">
+        <v>31</v>
+      </c>
+      <c r="S2" t="s">
+        <v>32</v>
+      </c>
+      <c r="T2" t="s">
+        <v>33</v>
+      </c>
+      <c r="U2" t="s">
+        <v>34</v>
+      </c>
+      <c r="V2">
+        <v>180</v>
+      </c>
+      <c r="W2">
+        <v>2624</v>
+      </c>
+      <c r="X2">
+        <v>1863</v>
+      </c>
+      <c r="Y2">
+        <v>0</v>
+      </c>
+      <c r="Z2" t="s">
+        <v>35</v>
+      </c>
+      <c r="AA2" t="s">
+        <v>36</v>
+      </c>
+      <c r="AB2" t="s">
+        <v>37</v>
+      </c>
+      <c r="AC2">
+        <v>0.196394831367994</v>
+      </c>
+      <c r="AD2">
+        <v>0.196394831367994</v>
       </c>
     </row>
   </sheetData>
@@ -1009,57 +1207,57 @@
   <sheetData>
     <row r="1" spans="1:16">
       <c r="A1" t="s">
-        <v>142</v>
+        <v>184</v>
       </c>
       <c r="B1" t="s">
-        <v>117</v>
+        <v>157</v>
       </c>
       <c r="C1" t="s">
-        <v>143</v>
+        <v>185</v>
       </c>
       <c r="D1" t="s">
-        <v>123</v>
+        <v>164</v>
       </c>
       <c r="E1" t="s">
-        <v>118</v>
+        <v>158</v>
       </c>
       <c r="F1" t="s">
-        <v>124</v>
+        <v>165</v>
       </c>
       <c r="G1" t="s">
-        <v>125</v>
+        <v>166</v>
       </c>
       <c r="H1" t="s">
-        <v>144</v>
+        <v>186</v>
       </c>
       <c r="I1" t="s">
-        <v>145</v>
+        <v>187</v>
       </c>
       <c r="J1" t="s">
-        <v>146</v>
+        <v>188</v>
       </c>
       <c r="K1" t="s">
-        <v>126</v>
+        <v>167</v>
       </c>
       <c r="L1" t="s">
-        <v>147</v>
+        <v>189</v>
       </c>
       <c r="M1" t="s">
-        <v>148</v>
+        <v>190</v>
       </c>
       <c r="N1" t="s">
-        <v>149</v>
+        <v>191</v>
       </c>
       <c r="O1" t="s">
-        <v>133</v>
+        <v>174</v>
       </c>
       <c r="P1" t="s">
-        <v>134</v>
+        <v>175</v>
       </c>
     </row>
     <row r="2" spans="1:16">
       <c r="A2" t="s">
-        <v>150</v>
+        <v>192</v>
       </c>
       <c r="B2">
         <v>75</v>
@@ -1109,7 +1307,7 @@
     </row>
     <row r="3" spans="1:16">
       <c r="A3" t="s">
-        <v>151</v>
+        <v>193</v>
       </c>
       <c r="B3">
         <v>27</v>
@@ -1159,7 +1357,7 @@
     </row>
     <row r="4" spans="1:16">
       <c r="A4" t="s">
-        <v>152</v>
+        <v>194</v>
       </c>
       <c r="B4">
         <v>38</v>
@@ -1209,7 +1407,7 @@
     </row>
     <row r="5" spans="1:16">
       <c r="A5" t="s">
-        <v>153</v>
+        <v>195</v>
       </c>
       <c r="B5">
         <v>62</v>
@@ -1259,7 +1457,7 @@
     </row>
     <row r="6" spans="1:16">
       <c r="A6" t="s">
-        <v>154</v>
+        <v>196</v>
       </c>
       <c r="B6">
         <v>56</v>
@@ -1309,7 +1507,7 @@
     </row>
     <row r="7" spans="1:16">
       <c r="A7" t="s">
-        <v>155</v>
+        <v>197</v>
       </c>
       <c r="B7">
         <v>56</v>
@@ -1359,7 +1557,7 @@
     </row>
     <row r="8" spans="1:16">
       <c r="A8" t="s">
-        <v>156</v>
+        <v>198</v>
       </c>
       <c r="B8">
         <v>55</v>
@@ -1409,7 +1607,7 @@
     </row>
     <row r="9" spans="1:16">
       <c r="A9" t="s">
-        <v>157</v>
+        <v>199</v>
       </c>
       <c r="B9">
         <v>57</v>
@@ -1459,7 +1657,7 @@
     </row>
     <row r="10" spans="1:16">
       <c r="A10" t="s">
-        <v>158</v>
+        <v>200</v>
       </c>
       <c r="B10">
         <v>84</v>
@@ -1509,7 +1707,7 @@
     </row>
     <row r="11" spans="1:16">
       <c r="A11" t="s">
-        <v>159</v>
+        <v>201</v>
       </c>
       <c r="B11">
         <v>86</v>
@@ -1559,7 +1757,7 @@
     </row>
     <row r="12" spans="1:16">
       <c r="A12" t="s">
-        <v>160</v>
+        <v>202</v>
       </c>
       <c r="B12">
         <v>108</v>
@@ -1609,7 +1807,7 @@
     </row>
     <row r="13" spans="1:16">
       <c r="A13" t="s">
-        <v>161</v>
+        <v>203</v>
       </c>
       <c r="B13">
         <v>92</v>
@@ -1659,7 +1857,7 @@
     </row>
     <row r="14" spans="1:16">
       <c r="A14" t="s">
-        <v>162</v>
+        <v>204</v>
       </c>
       <c r="B14">
         <v>68</v>
@@ -1709,7 +1907,7 @@
     </row>
     <row r="15" spans="1:16">
       <c r="A15" t="s">
-        <v>163</v>
+        <v>205</v>
       </c>
       <c r="B15">
         <v>90</v>
@@ -1759,7 +1957,7 @@
     </row>
     <row r="16" spans="1:16">
       <c r="A16" t="s">
-        <v>164</v>
+        <v>206</v>
       </c>
       <c r="B16">
         <v>86</v>
@@ -1809,7 +2007,7 @@
     </row>
     <row r="17" spans="1:16">
       <c r="A17" t="s">
-        <v>165</v>
+        <v>207</v>
       </c>
       <c r="B17">
         <v>102</v>
@@ -1859,7 +2057,7 @@
     </row>
     <row r="18" spans="1:16">
       <c r="A18" t="s">
-        <v>166</v>
+        <v>208</v>
       </c>
       <c r="B18">
         <v>134</v>
@@ -1909,7 +2107,7 @@
     </row>
     <row r="19" spans="1:16">
       <c r="A19" t="s">
-        <v>167</v>
+        <v>209</v>
       </c>
       <c r="B19">
         <v>124</v>
@@ -1959,10 +2157,10 @@
     </row>
     <row r="20" spans="1:16">
       <c r="A20" t="s">
-        <v>168</v>
+        <v>210</v>
       </c>
       <c r="B20">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C20">
         <v>155</v>
@@ -1977,13 +2175,13 @@
         <v>484440</v>
       </c>
       <c r="G20">
-        <v>7718.185185185185</v>
+        <v>7766.124223602485</v>
       </c>
       <c r="H20">
         <v>61</v>
       </c>
       <c r="I20">
-        <v>0.2901234567901235</v>
+        <v>0.2919254658385093</v>
       </c>
       <c r="J20">
         <v>0.3032258064516129</v>
@@ -1992,13 +2190,13 @@
         <v>0.3032258064516129</v>
       </c>
       <c r="L20">
-        <v>0.9567901234567902</v>
+        <v>0.9627329192546584</v>
       </c>
       <c r="M20" t="b">
         <v>1</v>
       </c>
       <c r="N20">
-        <v>0.3765432098765432</v>
+        <v>0.3788819875776397</v>
       </c>
       <c r="O20">
         <v>0.2363435226543088</v>
@@ -2009,16 +2207,16 @@
     </row>
     <row r="21" spans="1:16">
       <c r="A21" t="s">
-        <v>169</v>
+        <v>211</v>
       </c>
       <c r="B21">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C21">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="D21">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E21">
         <v>1313200</v>
@@ -2027,42 +2225,42 @@
         <v>457066</v>
       </c>
       <c r="G21">
-        <v>8417.948717948719</v>
+        <v>8472.258064516129</v>
       </c>
       <c r="H21">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="I21">
-        <v>0.2948717948717949</v>
+        <v>0.2903225806451613</v>
       </c>
       <c r="J21">
-        <v>0.3194444444444444</v>
+        <v>0.3146853146853147</v>
       </c>
       <c r="K21">
-        <v>0.3194444444444444</v>
+        <v>0.3146853146853147</v>
       </c>
       <c r="L21">
-        <v>0.9230769230769231</v>
+        <v>0.9225806451612903</v>
       </c>
       <c r="M21" t="b">
         <v>1</v>
       </c>
       <c r="N21">
-        <v>0.3076923076923077</v>
+        <v>0.3032258064516129</v>
       </c>
       <c r="O21">
-        <v>0.2488297377623892</v>
+        <v>0.2442641903306046</v>
       </c>
       <c r="P21">
-        <v>0.3994424670838787</v>
+        <v>0.3948026681073313</v>
       </c>
     </row>
     <row r="22" spans="1:16">
       <c r="A22" t="s">
-        <v>170</v>
+        <v>212</v>
       </c>
       <c r="B22">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C22">
         <v>160</v>
@@ -2077,13 +2275,13 @@
         <v>431339.79</v>
       </c>
       <c r="G22">
-        <v>8523.7951497006</v>
+        <v>8575.143313253013</v>
       </c>
       <c r="H22">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="I22">
-        <v>0.3173652694610778</v>
+        <v>0.3192771084337349</v>
       </c>
       <c r="J22">
         <v>0.33125</v>
@@ -2092,13 +2290,13 @@
         <v>0.33125</v>
       </c>
       <c r="L22">
-        <v>0.9580838323353293</v>
+        <v>0.963855421686747</v>
       </c>
       <c r="M22" t="b">
         <v>1</v>
       </c>
       <c r="N22">
-        <v>0.1976047904191617</v>
+        <v>0.1927710843373494</v>
       </c>
       <c r="O22">
         <v>0.2630282728403034</v>
@@ -2109,63 +2307,63 @@
     </row>
     <row r="23" spans="1:16">
       <c r="A23" t="s">
-        <v>171</v>
+        <v>213</v>
       </c>
       <c r="B23">
-        <v>179</v>
+        <v>172</v>
       </c>
       <c r="C23">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D23">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E23">
-        <v>1584444</v>
+        <v>1554444</v>
       </c>
       <c r="F23">
-        <v>205297</v>
+        <v>195297</v>
       </c>
       <c r="G23">
-        <v>8851.642458100559</v>
+        <v>9037.465116279071</v>
       </c>
       <c r="H23">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="I23">
-        <v>0.2681564245810056</v>
+        <v>0.2732558139534884</v>
       </c>
       <c r="J23">
-        <v>0.2807017543859649</v>
+        <v>0.2764705882352941</v>
       </c>
       <c r="K23">
-        <v>0.2807017543859649</v>
+        <v>0.2764705882352941</v>
       </c>
       <c r="L23">
-        <v>0.9553072625698324</v>
+        <v>0.9883720930232558</v>
       </c>
       <c r="M23" t="b">
         <v>1</v>
       </c>
       <c r="N23">
-        <v>0.223463687150838</v>
+        <v>0.2151162790697674</v>
       </c>
       <c r="O23">
-        <v>0.2187404908403237</v>
+        <v>0.2147407197533275</v>
       </c>
       <c r="P23">
-        <v>0.3522998107812584</v>
+        <v>0.3480796868697131</v>
       </c>
     </row>
     <row r="24" spans="1:16">
       <c r="A24" t="s">
-        <v>172</v>
+        <v>214</v>
       </c>
       <c r="B24">
-        <v>312</v>
+        <v>293</v>
       </c>
       <c r="C24">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="D24">
         <v>58</v>
@@ -2177,92 +2375,92 @@
         <v>523625</v>
       </c>
       <c r="G24">
-        <v>6869.05340909091</v>
+        <v>7220.7114334471</v>
       </c>
       <c r="H24">
-        <v>114</v>
+        <v>105</v>
       </c>
       <c r="I24">
-        <v>0.1858974358974359</v>
+        <v>0.1979522184300341</v>
       </c>
       <c r="J24">
-        <v>0.2301587301587301</v>
+        <v>0.2329317269076305</v>
       </c>
       <c r="K24">
-        <v>0.2301587301587301</v>
+        <v>0.2329317269076305</v>
       </c>
       <c r="L24">
-        <v>0.8076923076923077</v>
+        <v>0.8498293515358362</v>
       </c>
       <c r="M24" t="b">
         <v>1</v>
       </c>
       <c r="N24">
-        <v>0.3653846153846154</v>
+        <v>0.3583617747440273</v>
       </c>
       <c r="O24">
-        <v>0.1824712333379016</v>
+        <v>0.1847286645878152</v>
       </c>
       <c r="P24">
-        <v>0.2859498522087804</v>
+        <v>0.2892503008988768</v>
       </c>
     </row>
     <row r="25" spans="1:16">
       <c r="A25" t="s">
-        <v>173</v>
+        <v>215</v>
       </c>
       <c r="B25">
-        <v>291</v>
+        <v>281</v>
       </c>
       <c r="C25">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="D25">
         <v>56</v>
       </c>
       <c r="E25">
-        <v>3506242.05</v>
+        <v>3436242.05</v>
       </c>
       <c r="F25">
         <v>381088.44</v>
       </c>
       <c r="G25">
-        <v>12048.94175257732</v>
+        <v>12228.61939501779</v>
       </c>
       <c r="H25">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="I25">
-        <v>0.1924398625429553</v>
+        <v>0.199288256227758</v>
       </c>
       <c r="J25">
-        <v>0.21875</v>
+        <v>0.2196078431372549</v>
       </c>
       <c r="K25">
-        <v>0.21875</v>
+        <v>0.2196078431372549</v>
       </c>
       <c r="L25">
-        <v>0.8797250859106529</v>
+        <v>0.9074733096085409</v>
       </c>
       <c r="M25" t="b">
         <v>1</v>
       </c>
       <c r="N25">
-        <v>0.2302405498281787</v>
+        <v>0.2277580071174377</v>
       </c>
       <c r="O25">
-        <v>0.172470829071034</v>
+        <v>0.1731643553495858</v>
       </c>
       <c r="P25">
-        <v>0.2733453912724368</v>
+        <v>0.2743742165028521</v>
       </c>
     </row>
     <row r="26" spans="1:16">
       <c r="A26" t="s">
-        <v>174</v>
+        <v>216</v>
       </c>
       <c r="B26">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="C26">
         <v>223</v>
@@ -2271,19 +2469,19 @@
         <v>63</v>
       </c>
       <c r="E26">
-        <v>3909935.66</v>
+        <v>3875742.16</v>
       </c>
       <c r="F26">
         <v>484712.91</v>
       </c>
       <c r="G26">
-        <v>12694.5962987013</v>
+        <v>12665.82405228758</v>
       </c>
       <c r="H26">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="I26">
-        <v>0.2045454545454546</v>
+        <v>0.2058823529411765</v>
       </c>
       <c r="J26">
         <v>0.2825112107623318</v>
@@ -2292,13 +2490,13 @@
         <v>0.2825112107623318</v>
       </c>
       <c r="L26">
-        <v>0.724025974025974</v>
+        <v>0.7287581699346405</v>
       </c>
       <c r="M26" t="b">
         <v>0</v>
       </c>
       <c r="N26">
-        <v>0.1136363636363636</v>
+        <v>0.107843137254902</v>
       </c>
       <c r="O26">
         <v>0.2274892170515385</v>
@@ -2309,16 +2507,16 @@
     </row>
     <row r="27" spans="1:16">
       <c r="A27" t="s">
-        <v>175</v>
+        <v>217</v>
       </c>
       <c r="B27">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="C27">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D27">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E27">
         <v>4789095.36</v>
@@ -2327,34 +2525,34 @@
         <v>249992.29</v>
       </c>
       <c r="G27">
-        <v>15300.62415335463</v>
+        <v>15399.02045016077</v>
       </c>
       <c r="H27">
         <v>21</v>
       </c>
       <c r="I27">
-        <v>0.1501597444089457</v>
+        <v>0.1479099678456592</v>
       </c>
       <c r="J27">
-        <v>0.4051724137931034</v>
+        <v>0.4</v>
       </c>
       <c r="K27">
-        <v>0.4051724137931034</v>
+        <v>0.4</v>
       </c>
       <c r="L27">
-        <v>0.3706070287539936</v>
+        <v>0.3697749196141479</v>
       </c>
       <c r="M27" t="b">
         <v>0</v>
       </c>
       <c r="N27">
-        <v>0.0670926517571885</v>
+        <v>0.06752411575562701</v>
       </c>
       <c r="O27">
-        <v>0.3202639001453139</v>
+        <v>0.3150932123418453</v>
       </c>
       <c r="P27">
-        <v>0.4961604466591346</v>
+        <v>0.4913718638604273</v>
       </c>
     </row>
   </sheetData>
@@ -2364,109 +2562,71 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:10">
       <c r="A1" t="s">
-        <v>20</v>
+        <v>38</v>
       </c>
       <c r="B1" t="s">
-        <v>21</v>
+        <v>39</v>
       </c>
       <c r="C1" t="s">
-        <v>22</v>
+        <v>40</v>
       </c>
       <c r="D1" t="s">
-        <v>23</v>
+        <v>41</v>
       </c>
       <c r="E1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5">
+        <v>42</v>
+      </c>
+      <c r="F1" t="s">
+        <v>43</v>
+      </c>
+      <c r="G1" t="s">
+        <v>44</v>
+      </c>
+      <c r="H1" t="s">
+        <v>45</v>
+      </c>
+      <c r="I1" t="s">
+        <v>46</v>
+      </c>
+      <c r="J1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10">
       <c r="A2" t="s">
-        <v>25</v>
+        <v>48</v>
       </c>
       <c r="B2">
-        <v>114</v>
+        <v>430</v>
       </c>
       <c r="C2">
-        <v>0.157416413880665</v>
+        <v>100</v>
       </c>
       <c r="D2">
-        <v>0.1578947368421053</v>
+        <v>0.4289529709028777</v>
       </c>
       <c r="E2">
-        <v>0.000478322961440264</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5">
-      <c r="A3" t="s">
-        <v>26</v>
-      </c>
-      <c r="B3">
-        <v>114</v>
-      </c>
-      <c r="C3">
-        <v>0.2375058115393008</v>
-      </c>
-      <c r="D3">
-        <v>0.1666666666666667</v>
-      </c>
-      <c r="E3">
-        <v>0.07083914487263418</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5">
-      <c r="A4" t="s">
-        <v>27</v>
-      </c>
-      <c r="B4">
-        <v>113</v>
-      </c>
-      <c r="C4">
-        <v>0.325040471622965</v>
-      </c>
-      <c r="D4">
-        <v>0.2123893805309734</v>
-      </c>
-      <c r="E4">
-        <v>0.1126510910919915</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5">
-      <c r="A5" t="s">
-        <v>28</v>
-      </c>
-      <c r="B5">
-        <v>114</v>
-      </c>
-      <c r="C5">
-        <v>0.4113530808383302</v>
-      </c>
-      <c r="D5">
-        <v>0.2719298245614035</v>
-      </c>
-      <c r="E5">
-        <v>0.1394232562769266</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5">
-      <c r="A6" t="s">
-        <v>29</v>
-      </c>
-      <c r="B6">
-        <v>114</v>
-      </c>
-      <c r="C6">
-        <v>0.6105696005475619</v>
-      </c>
-      <c r="D6">
-        <v>0.6140350877192983</v>
-      </c>
-      <c r="E6">
-        <v>0.003465487171736337</v>
+        <v>0.2325581395348837</v>
+      </c>
+      <c r="F2">
+        <v>0.4284564457706168</v>
+      </c>
+      <c r="G2">
+        <v>0.4295981880533556</v>
+      </c>
+      <c r="H2">
+        <v>0.1951019908211038</v>
+      </c>
+      <c r="I2">
+        <v>0.2747506005394296</v>
+      </c>
+      <c r="J2">
+        <v>0.196394831367994</v>
       </c>
     </row>
   </sheetData>
@@ -2476,55 +2636,31 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
-        <v>30</v>
+        <v>49</v>
       </c>
       <c r="B1" t="s">
-        <v>31</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>32</v>
+        <v>51</v>
       </c>
       <c r="B2">
-        <v>0.5096243532884293</v>
+        <v>0.863918765539113</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>33</v>
+        <v>52</v>
       </c>
       <c r="B3">
-        <v>0.2047727006722439</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2">
-      <c r="A4" t="s">
-        <v>34</v>
-      </c>
-      <c r="B4">
-        <v>0.141902655441849</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2">
-      <c r="A5" t="s">
-        <v>35</v>
-      </c>
-      <c r="B5">
-        <v>0.1054955021512117</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2">
-      <c r="A6" t="s">
-        <v>36</v>
-      </c>
-      <c r="B6">
-        <v>0.03820478844626608</v>
+        <v>0.1360812344608871</v>
       </c>
     </row>
   </sheetData>
@@ -2534,553 +2670,595 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:9">
       <c r="A1" t="s">
-        <v>37</v>
+        <v>53</v>
       </c>
       <c r="B1" t="s">
-        <v>38</v>
+        <v>54</v>
       </c>
       <c r="C1" t="s">
-        <v>39</v>
+        <v>55</v>
       </c>
       <c r="D1" t="s">
-        <v>33</v>
+        <v>56</v>
       </c>
       <c r="E1" t="s">
-        <v>32</v>
+        <v>57</v>
       </c>
       <c r="F1" t="s">
-        <v>35</v>
+        <v>58</v>
       </c>
       <c r="G1" t="s">
-        <v>40</v>
+        <v>59</v>
       </c>
       <c r="H1" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8">
+        <v>60</v>
+      </c>
+      <c r="I1" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
       <c r="A2" t="s">
-        <v>42</v>
+        <v>62</v>
       </c>
       <c r="B2" t="s">
-        <v>62</v>
+        <v>82</v>
       </c>
       <c r="C2" t="s">
+        <v>101</v>
+      </c>
+      <c r="D2">
+        <v>20000</v>
+      </c>
+      <c r="E2" t="s">
+        <v>103</v>
+      </c>
+      <c r="G2">
+        <v>0.7300433547112769</v>
+      </c>
+      <c r="H2" t="s">
+        <v>110</v>
+      </c>
+      <c r="I2" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9">
+      <c r="A3" t="s">
+        <v>63</v>
+      </c>
+      <c r="B3" t="s">
+        <v>83</v>
+      </c>
+      <c r="C3" t="s">
+        <v>101</v>
+      </c>
+      <c r="D3">
+        <v>20000</v>
+      </c>
+      <c r="E3" t="s">
+        <v>103</v>
+      </c>
+      <c r="G3">
+        <v>0.7300433547112769</v>
+      </c>
+      <c r="H3" t="s">
+        <v>110</v>
+      </c>
+      <c r="I3" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9">
+      <c r="A4" t="s">
+        <v>64</v>
+      </c>
+      <c r="B4" t="s">
+        <v>84</v>
+      </c>
+      <c r="C4" t="s">
+        <v>101</v>
+      </c>
+      <c r="D4">
+        <v>20000</v>
+      </c>
+      <c r="E4" t="s">
+        <v>103</v>
+      </c>
+      <c r="F4" t="s">
+        <v>108</v>
+      </c>
+      <c r="G4">
+        <v>0.7300433547112769</v>
+      </c>
+      <c r="H4" t="s">
+        <v>110</v>
+      </c>
+      <c r="I4" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
+      <c r="A5" t="s">
+        <v>65</v>
+      </c>
+      <c r="B5" t="s">
+        <v>85</v>
+      </c>
+      <c r="C5" t="s">
+        <v>101</v>
+      </c>
+      <c r="D5">
+        <v>20000</v>
+      </c>
+      <c r="E5" t="s">
+        <v>103</v>
+      </c>
+      <c r="F5" t="s">
+        <v>109</v>
+      </c>
+      <c r="G5">
+        <v>0.7300433547112769</v>
+      </c>
+      <c r="H5" t="s">
+        <v>110</v>
+      </c>
+      <c r="I5" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9">
+      <c r="A6" t="s">
+        <v>66</v>
+      </c>
+      <c r="B6" t="s">
+        <v>86</v>
+      </c>
+      <c r="C6" t="s">
+        <v>101</v>
+      </c>
+      <c r="D6">
+        <v>20000</v>
+      </c>
+      <c r="E6" t="s">
+        <v>103</v>
+      </c>
+      <c r="G6">
+        <v>0.6801311886649636</v>
+      </c>
+      <c r="H6" t="s">
+        <v>110</v>
+      </c>
+      <c r="I6" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9">
+      <c r="A7" t="s">
+        <v>67</v>
+      </c>
+      <c r="B7" t="s">
+        <v>87</v>
+      </c>
+      <c r="C7" t="s">
+        <v>101</v>
+      </c>
+      <c r="D7">
+        <v>20000</v>
+      </c>
+      <c r="E7" t="s">
+        <v>103</v>
+      </c>
+      <c r="G7">
+        <v>0.6801311886649636</v>
+      </c>
+      <c r="H7" t="s">
+        <v>110</v>
+      </c>
+      <c r="I7" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9">
+      <c r="A8" t="s">
+        <v>68</v>
+      </c>
+      <c r="B8" t="s">
+        <v>88</v>
+      </c>
+      <c r="C8" t="s">
+        <v>101</v>
+      </c>
+      <c r="D8">
+        <v>31829</v>
+      </c>
+      <c r="E8" t="s">
+        <v>103</v>
+      </c>
+      <c r="F8" t="s">
+        <v>108</v>
+      </c>
+      <c r="G8">
+        <v>0.6691801734898181</v>
+      </c>
+      <c r="H8" t="s">
+        <v>110</v>
+      </c>
+      <c r="I8" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9">
+      <c r="A9" t="s">
+        <v>69</v>
+      </c>
+      <c r="B9" t="s">
+        <v>89</v>
+      </c>
+      <c r="C9" t="s">
+        <v>101</v>
+      </c>
+      <c r="D9">
+        <v>20000</v>
+      </c>
+      <c r="E9" t="s">
+        <v>104</v>
+      </c>
+      <c r="G9">
+        <v>0.6691801734898181</v>
+      </c>
+      <c r="H9" t="s">
+        <v>110</v>
+      </c>
+      <c r="I9" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9">
+      <c r="A10" t="s">
+        <v>70</v>
+      </c>
+      <c r="B10" t="s">
+        <v>90</v>
+      </c>
+      <c r="C10" t="s">
+        <v>101</v>
+      </c>
+      <c r="D10">
+        <v>20000</v>
+      </c>
+      <c r="E10" t="s">
+        <v>105</v>
+      </c>
+      <c r="F10" t="s">
+        <v>108</v>
+      </c>
+      <c r="G10">
+        <v>0.6691801734898181</v>
+      </c>
+      <c r="H10" t="s">
+        <v>110</v>
+      </c>
+      <c r="I10" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9">
+      <c r="A11" t="s">
+        <v>71</v>
+      </c>
+      <c r="B11" t="s">
+        <v>91</v>
+      </c>
+      <c r="C11" t="s">
+        <v>101</v>
+      </c>
+      <c r="D11">
+        <v>19655</v>
+      </c>
+      <c r="E11" t="s">
+        <v>106</v>
+      </c>
+      <c r="F11" t="s">
+        <v>108</v>
+      </c>
+      <c r="G11">
+        <v>0.6691801734898181</v>
+      </c>
+      <c r="H11" t="s">
+        <v>110</v>
+      </c>
+      <c r="I11" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9">
+      <c r="A12" t="s">
+        <v>72</v>
+      </c>
+      <c r="B12" t="s">
+        <v>92</v>
+      </c>
+      <c r="C12" t="s">
+        <v>101</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+      <c r="E12" t="s">
+        <v>105</v>
+      </c>
+      <c r="F12" t="s">
+        <v>108</v>
+      </c>
+      <c r="G12">
+        <v>0.6691801734898181</v>
+      </c>
+      <c r="H12" t="s">
+        <v>110</v>
+      </c>
+      <c r="I12" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9">
+      <c r="A13" t="s">
+        <v>73</v>
+      </c>
+      <c r="B13" t="s">
+        <v>93</v>
+      </c>
+      <c r="C13" t="s">
+        <v>101</v>
+      </c>
+      <c r="D13">
+        <v>21136</v>
+      </c>
+      <c r="E13" t="s">
+        <v>103</v>
+      </c>
+      <c r="F13" t="s">
+        <v>108</v>
+      </c>
+      <c r="G13">
+        <v>0.653900255242338</v>
+      </c>
+      <c r="H13" t="s">
+        <v>110</v>
+      </c>
+      <c r="I13" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9">
+      <c r="A14" t="s">
+        <v>74</v>
+      </c>
+      <c r="B14" t="s">
+        <v>94</v>
+      </c>
+      <c r="C14" t="s">
+        <v>101</v>
+      </c>
+      <c r="D14">
+        <v>20000</v>
+      </c>
+      <c r="E14" t="s">
+        <v>103</v>
+      </c>
+      <c r="G14">
+        <v>0.653900255242338</v>
+      </c>
+      <c r="H14" t="s">
+        <v>110</v>
+      </c>
+      <c r="I14" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9">
+      <c r="A15" t="s">
+        <v>75</v>
+      </c>
+      <c r="B15" t="s">
+        <v>95</v>
+      </c>
+      <c r="C15" t="s">
+        <v>101</v>
+      </c>
+      <c r="D15">
+        <v>20000</v>
+      </c>
+      <c r="E15" t="s">
+        <v>105</v>
+      </c>
+      <c r="G15">
+        <v>0.653900255242338</v>
+      </c>
+      <c r="H15" t="s">
+        <v>110</v>
+      </c>
+      <c r="I15" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9">
+      <c r="A16" t="s">
         <v>76</v>
       </c>
-      <c r="D2">
-        <v>31829</v>
-      </c>
-      <c r="E2" t="s">
+      <c r="B16" t="s">
+        <v>96</v>
+      </c>
+      <c r="C16" t="s">
+        <v>101</v>
+      </c>
+      <c r="D16">
+        <v>21803</v>
+      </c>
+      <c r="E16" t="s">
+        <v>103</v>
+      </c>
+      <c r="F16" t="s">
+        <v>108</v>
+      </c>
+      <c r="G16">
+        <v>0.6527051193075826</v>
+      </c>
+      <c r="H16" t="s">
+        <v>110</v>
+      </c>
+      <c r="I16" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9">
+      <c r="A17" t="s">
+        <v>77</v>
+      </c>
+      <c r="B17" t="s">
+        <v>84</v>
+      </c>
+      <c r="C17" t="s">
+        <v>101</v>
+      </c>
+      <c r="D17">
+        <v>20000</v>
+      </c>
+      <c r="E17" t="s">
+        <v>107</v>
+      </c>
+      <c r="F17" t="s">
+        <v>108</v>
+      </c>
+      <c r="G17">
+        <v>0.6527051193075826</v>
+      </c>
+      <c r="H17" t="s">
+        <v>110</v>
+      </c>
+      <c r="I17" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9">
+      <c r="A18" t="s">
+        <v>78</v>
+      </c>
+      <c r="B18" t="s">
+        <v>97</v>
+      </c>
+      <c r="C18" t="s">
+        <v>101</v>
+      </c>
+      <c r="D18">
+        <v>20000</v>
+      </c>
+      <c r="E18" t="s">
+        <v>103</v>
+      </c>
+      <c r="F18" t="s">
+        <v>108</v>
+      </c>
+      <c r="G18">
+        <v>0.6527051193075826</v>
+      </c>
+      <c r="H18" t="s">
+        <v>110</v>
+      </c>
+      <c r="I18" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9">
+      <c r="A19" t="s">
+        <v>79</v>
+      </c>
+      <c r="B19" t="s">
+        <v>98</v>
+      </c>
+      <c r="C19" t="s">
+        <v>101</v>
+      </c>
+      <c r="D19">
+        <v>20000</v>
+      </c>
+      <c r="E19" t="s">
+        <v>105</v>
+      </c>
+      <c r="F19" t="s">
+        <v>108</v>
+      </c>
+      <c r="G19">
+        <v>0.6527051193075826</v>
+      </c>
+      <c r="H19" t="s">
+        <v>110</v>
+      </c>
+      <c r="I19" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9">
+      <c r="A20" t="s">
+        <v>80</v>
+      </c>
+      <c r="B20" t="s">
+        <v>99</v>
+      </c>
+      <c r="C20" t="s">
+        <v>101</v>
+      </c>
+      <c r="D20">
+        <v>10000</v>
+      </c>
+      <c r="E20" t="s">
+        <v>105</v>
+      </c>
+      <c r="F20" t="s">
+        <v>108</v>
+      </c>
+      <c r="G20">
+        <v>0.6527051193075826</v>
+      </c>
+      <c r="H20" t="s">
+        <v>110</v>
+      </c>
+      <c r="I20" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9">
+      <c r="A21" t="s">
         <v>81</v>
       </c>
-      <c r="F2" t="s">
-        <v>83</v>
-      </c>
-      <c r="G2">
-        <v>0.7733831110668795</v>
-      </c>
-      <c r="H2" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8">
-      <c r="A3" t="s">
-        <v>43</v>
-      </c>
-      <c r="B3" t="s">
-        <v>63</v>
-      </c>
-      <c r="C3" t="s">
-        <v>76</v>
-      </c>
-      <c r="D3">
-        <v>21136</v>
-      </c>
-      <c r="E3" t="s">
-        <v>81</v>
-      </c>
-      <c r="F3" t="s">
-        <v>83</v>
-      </c>
-      <c r="G3">
-        <v>0.7584242825937598</v>
-      </c>
-      <c r="H3" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8">
-      <c r="A4" t="s">
-        <v>44</v>
-      </c>
-      <c r="B4" t="s">
-        <v>64</v>
-      </c>
-      <c r="C4" t="s">
-        <v>77</v>
-      </c>
-      <c r="D4">
-        <v>372.61</v>
-      </c>
-      <c r="E4" t="s">
-        <v>82</v>
-      </c>
-      <c r="F4" t="s">
-        <v>84</v>
-      </c>
-      <c r="G4">
-        <v>0.7573678487216609</v>
-      </c>
-      <c r="H4" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8">
-      <c r="A5" t="s">
-        <v>45</v>
-      </c>
-      <c r="B5" t="s">
-        <v>65</v>
-      </c>
-      <c r="C5" t="s">
-        <v>78</v>
-      </c>
-      <c r="D5">
-        <v>327.93</v>
-      </c>
-      <c r="E5" t="s">
-        <v>82</v>
-      </c>
-      <c r="F5" t="s">
-        <v>84</v>
-      </c>
-      <c r="G5">
-        <v>0.7430330869295462</v>
-      </c>
-      <c r="H5" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8">
-      <c r="A6" t="s">
-        <v>46</v>
-      </c>
-      <c r="B6" t="s">
-        <v>66</v>
-      </c>
-      <c r="C6" t="s">
-        <v>77</v>
-      </c>
-      <c r="D6">
-        <v>62</v>
-      </c>
-      <c r="E6" t="s">
-        <v>82</v>
-      </c>
-      <c r="F6" t="s">
-        <v>84</v>
-      </c>
-      <c r="G6">
-        <v>0.7410267602055233</v>
-      </c>
-      <c r="H6" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8">
-      <c r="A7" t="s">
-        <v>47</v>
-      </c>
-      <c r="B7" t="s">
-        <v>67</v>
-      </c>
-      <c r="C7" t="s">
-        <v>79</v>
-      </c>
-      <c r="D7">
-        <v>0</v>
-      </c>
-      <c r="E7" t="s">
-        <v>82</v>
-      </c>
-      <c r="F7" t="s">
-        <v>83</v>
-      </c>
-      <c r="G7">
-        <v>0.7408532634654529</v>
-      </c>
-      <c r="H7" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8">
-      <c r="A8" t="s">
-        <v>48</v>
-      </c>
-      <c r="B8" t="s">
-        <v>65</v>
-      </c>
-      <c r="C8" t="s">
-        <v>78</v>
-      </c>
-      <c r="D8">
-        <v>111.5</v>
-      </c>
-      <c r="E8" t="s">
-        <v>82</v>
-      </c>
-      <c r="F8" t="s">
-        <v>84</v>
-      </c>
-      <c r="G8">
-        <v>0.7405346644903105</v>
-      </c>
-      <c r="H8" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8">
-      <c r="A9" t="s">
-        <v>49</v>
-      </c>
-      <c r="B9" t="s">
-        <v>68</v>
-      </c>
-      <c r="C9" t="s">
-        <v>80</v>
-      </c>
-      <c r="D9">
-        <v>963</v>
-      </c>
-      <c r="E9" t="s">
-        <v>82</v>
-      </c>
-      <c r="F9" t="s">
-        <v>83</v>
-      </c>
-      <c r="G9">
-        <v>0.7391946960238088</v>
-      </c>
-      <c r="H9" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8">
-      <c r="A10" t="s">
-        <v>50</v>
-      </c>
-      <c r="B10" t="s">
-        <v>69</v>
-      </c>
-      <c r="C10" t="s">
-        <v>78</v>
-      </c>
-      <c r="D10">
-        <v>165</v>
-      </c>
-      <c r="E10" t="s">
-        <v>82</v>
-      </c>
-      <c r="F10" t="s">
-        <v>84</v>
-      </c>
-      <c r="G10">
-        <v>0.7391186414334949</v>
-      </c>
-      <c r="H10" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8">
-      <c r="A11" t="s">
-        <v>51</v>
-      </c>
-      <c r="B11" t="s">
-        <v>70</v>
-      </c>
-      <c r="C11" t="s">
-        <v>77</v>
-      </c>
-      <c r="D11">
-        <v>1092</v>
-      </c>
-      <c r="E11" t="s">
-        <v>82</v>
-      </c>
-      <c r="F11" t="s">
-        <v>84</v>
-      </c>
-      <c r="G11">
-        <v>0.7338072971228526</v>
-      </c>
-      <c r="H11" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8">
-      <c r="A12" t="s">
-        <v>52</v>
-      </c>
-      <c r="B12" t="s">
-        <v>71</v>
-      </c>
-      <c r="C12" t="s">
-        <v>80</v>
-      </c>
-      <c r="D12">
-        <v>1839</v>
-      </c>
-      <c r="E12" t="s">
-        <v>82</v>
-      </c>
-      <c r="F12" t="s">
-        <v>84</v>
-      </c>
-      <c r="G12">
-        <v>0.7222770753936161</v>
-      </c>
-      <c r="H12" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8">
-      <c r="A13" t="s">
-        <v>53</v>
-      </c>
-      <c r="B13" t="s">
-        <v>72</v>
-      </c>
-      <c r="C13" t="s">
-        <v>80</v>
-      </c>
-      <c r="D13">
-        <v>0</v>
-      </c>
-      <c r="E13" t="s">
-        <v>82</v>
-      </c>
-      <c r="F13" t="s">
-        <v>85</v>
-      </c>
-      <c r="G13">
-        <v>0.7166722139896516</v>
-      </c>
-      <c r="H13" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8">
-      <c r="A14" t="s">
-        <v>54</v>
-      </c>
-      <c r="B14" t="s">
-        <v>67</v>
-      </c>
-      <c r="C14" t="s">
-        <v>77</v>
-      </c>
-      <c r="D14">
-        <v>0</v>
-      </c>
-      <c r="E14" t="s">
-        <v>82</v>
-      </c>
-      <c r="F14" t="s">
-        <v>83</v>
-      </c>
-      <c r="G14">
-        <v>0.7085438876638861</v>
-      </c>
-      <c r="H14" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8">
-      <c r="A15" t="s">
-        <v>55</v>
-      </c>
-      <c r="B15" t="s">
-        <v>73</v>
-      </c>
-      <c r="C15" t="s">
-        <v>80</v>
-      </c>
-      <c r="D15">
-        <v>0</v>
-      </c>
-      <c r="E15" t="s">
-        <v>82</v>
-      </c>
-      <c r="F15" t="s">
-        <v>84</v>
-      </c>
-      <c r="G15">
-        <v>0.70356759914406</v>
-      </c>
-      <c r="H15" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8">
-      <c r="A16" t="s">
-        <v>56</v>
-      </c>
-      <c r="B16" t="s">
-        <v>73</v>
-      </c>
-      <c r="C16" t="s">
-        <v>80</v>
-      </c>
-      <c r="D16">
-        <v>0</v>
-      </c>
-      <c r="E16" t="s">
-        <v>82</v>
-      </c>
-      <c r="F16" t="s">
-        <v>84</v>
-      </c>
-      <c r="G16">
-        <v>0.70356759914406</v>
-      </c>
-      <c r="H16" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8">
-      <c r="A17" t="s">
-        <v>57</v>
-      </c>
-      <c r="B17" t="s">
-        <v>73</v>
-      </c>
-      <c r="C17" t="s">
-        <v>76</v>
-      </c>
-      <c r="D17">
-        <v>0</v>
-      </c>
-      <c r="E17" t="s">
-        <v>82</v>
-      </c>
-      <c r="F17" t="s">
-        <v>84</v>
-      </c>
-      <c r="G17">
-        <v>0.7016406634623601</v>
-      </c>
-      <c r="H17" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8">
-      <c r="A18" t="s">
-        <v>58</v>
-      </c>
-      <c r="B18" t="s">
-        <v>74</v>
-      </c>
-      <c r="C18" t="s">
-        <v>78</v>
-      </c>
-      <c r="D18">
-        <v>0</v>
-      </c>
-      <c r="E18" t="s">
-        <v>82</v>
-      </c>
-      <c r="F18" t="s">
-        <v>84</v>
-      </c>
-      <c r="G18">
-        <v>0.7016406634623601</v>
-      </c>
-      <c r="H18" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8">
-      <c r="A19" t="s">
-        <v>59</v>
-      </c>
-      <c r="B19" t="s">
-        <v>75</v>
-      </c>
-      <c r="C19" t="s">
-        <v>77</v>
-      </c>
-      <c r="D19">
-        <v>0</v>
-      </c>
-      <c r="E19" t="s">
-        <v>82</v>
-      </c>
-      <c r="F19" t="s">
-        <v>84</v>
-      </c>
-      <c r="G19">
-        <v>0.7016406634623601</v>
-      </c>
-      <c r="H19" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8">
-      <c r="A20" t="s">
-        <v>60</v>
-      </c>
-      <c r="B20" t="s">
-        <v>73</v>
-      </c>
-      <c r="C20" t="s">
-        <v>76</v>
-      </c>
-      <c r="D20">
-        <v>0</v>
-      </c>
-      <c r="E20" t="s">
-        <v>82</v>
-      </c>
-      <c r="F20" t="s">
-        <v>84</v>
-      </c>
-      <c r="G20">
-        <v>0.7016406634623601</v>
-      </c>
-      <c r="H20" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8">
-      <c r="A21" t="s">
-        <v>61</v>
-      </c>
       <c r="B21" t="s">
-        <v>73</v>
+        <v>100</v>
       </c>
       <c r="C21" t="s">
-        <v>76</v>
+        <v>102</v>
       </c>
       <c r="D21">
         <v>0</v>
       </c>
       <c r="E21" t="s">
-        <v>82</v>
+        <v>107</v>
       </c>
       <c r="F21" t="s">
-        <v>84</v>
+        <v>109</v>
       </c>
       <c r="G21">
-        <v>0.7016406634623601</v>
+        <v>0.6527051193075826</v>
       </c>
       <c r="H21" t="s">
-        <v>87</v>
+        <v>110</v>
+      </c>
+      <c r="I21" t="s">
+        <v>112</v>
       </c>
     </row>
   </sheetData>
@@ -3090,41 +3268,65 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:Q5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:17">
       <c r="A1" t="s">
-        <v>88</v>
+        <v>113</v>
       </c>
       <c r="B1" t="s">
-        <v>89</v>
+        <v>114</v>
       </c>
       <c r="C1" t="s">
-        <v>90</v>
+        <v>115</v>
       </c>
       <c r="D1" t="s">
-        <v>91</v>
+        <v>116</v>
       </c>
       <c r="E1" t="s">
-        <v>92</v>
+        <v>117</v>
       </c>
       <c r="F1" t="s">
-        <v>93</v>
+        <v>118</v>
       </c>
       <c r="G1" t="s">
-        <v>94</v>
+        <v>119</v>
       </c>
       <c r="H1" t="s">
-        <v>95</v>
+        <v>120</v>
       </c>
       <c r="I1" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9">
+        <v>121</v>
+      </c>
+      <c r="J1" t="s">
+        <v>122</v>
+      </c>
+      <c r="K1" t="s">
+        <v>123</v>
+      </c>
+      <c r="L1" t="s">
+        <v>124</v>
+      </c>
+      <c r="M1" t="s">
+        <v>125</v>
+      </c>
+      <c r="N1" t="s">
+        <v>126</v>
+      </c>
+      <c r="O1" t="s">
+        <v>127</v>
+      </c>
+      <c r="P1" t="s">
+        <v>128</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17">
       <c r="A2" t="s">
-        <v>97</v>
+        <v>130</v>
       </c>
       <c r="B2">
         <v>283</v>
@@ -3133,7 +3335,7 @@
         <v>81</v>
       </c>
       <c r="D2">
-        <v>0.05899520533666875</v>
+        <v>0.05925460636515913</v>
       </c>
       <c r="E2">
         <v>0.2862190812720848</v>
@@ -3145,97 +3347,193 @@
         <v>0.3414683332932292</v>
       </c>
       <c r="H2" t="s">
-        <v>101</v>
+        <v>134</v>
       </c>
       <c r="I2" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9">
+        <v>135</v>
+      </c>
+      <c r="J2" t="s">
+        <v>136</v>
+      </c>
+      <c r="K2" t="s">
+        <v>137</v>
+      </c>
+      <c r="L2" t="s">
+        <v>138</v>
+      </c>
+      <c r="M2" t="s">
+        <v>139</v>
+      </c>
+      <c r="N2" t="s">
+        <v>140</v>
+      </c>
+      <c r="O2" t="s">
+        <v>141</v>
+      </c>
+      <c r="P2" t="s">
+        <v>142</v>
+      </c>
+      <c r="Q2">
+        <v>0.2862190812720848</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17">
       <c r="A3" t="s">
-        <v>98</v>
+        <v>131</v>
       </c>
       <c r="B3">
         <v>526</v>
       </c>
       <c r="C3">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="D3">
-        <v>0.1096518657494267</v>
+        <v>0.1101340033500837</v>
       </c>
       <c r="E3">
-        <v>0.4258555133079848</v>
+        <v>0.4239543726235742</v>
       </c>
       <c r="F3">
-        <v>0.3842855257703783</v>
+        <v>0.3824225808962795</v>
       </c>
       <c r="G3">
-        <v>0.4685006654233671</v>
+        <v>0.4665888972511518</v>
       </c>
       <c r="H3" t="s">
-        <v>101</v>
+        <v>134</v>
       </c>
       <c r="I3" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9">
+        <v>135</v>
+      </c>
+      <c r="J3" t="s">
+        <v>136</v>
+      </c>
+      <c r="K3" t="s">
+        <v>137</v>
+      </c>
+      <c r="L3" t="s">
+        <v>138</v>
+      </c>
+      <c r="M3" t="s">
+        <v>139</v>
+      </c>
+      <c r="N3" t="s">
+        <v>140</v>
+      </c>
+      <c r="O3" t="s">
+        <v>141</v>
+      </c>
+      <c r="P3" t="s">
+        <v>142</v>
+      </c>
+      <c r="Q3">
+        <v>0.4239543726235742</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17">
       <c r="A4" t="s">
-        <v>99</v>
+        <v>132</v>
       </c>
       <c r="B4">
-        <v>732</v>
+        <v>735</v>
       </c>
       <c r="C4">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="D4">
-        <v>0.1525953721075672</v>
+        <v>0.153894472361809</v>
       </c>
       <c r="E4">
-        <v>0.459016393442623</v>
+        <v>0.4557823129251701</v>
       </c>
       <c r="F4">
-        <v>0.4232241202659477</v>
+        <v>0.4200990011376739</v>
       </c>
       <c r="G4">
-        <v>0.4952365919308077</v>
+        <v>0.4919254436147601</v>
       </c>
       <c r="H4" t="s">
-        <v>101</v>
+        <v>134</v>
       </c>
       <c r="I4" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9">
+        <v>135</v>
+      </c>
+      <c r="J4" t="s">
+        <v>136</v>
+      </c>
+      <c r="K4" t="s">
+        <v>137</v>
+      </c>
+      <c r="L4" t="s">
+        <v>138</v>
+      </c>
+      <c r="M4" t="s">
+        <v>139</v>
+      </c>
+      <c r="N4" t="s">
+        <v>140</v>
+      </c>
+      <c r="O4" t="s">
+        <v>141</v>
+      </c>
+      <c r="P4" t="s">
+        <v>142</v>
+      </c>
+      <c r="Q4">
+        <v>0.4557823129251701</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17">
       <c r="A5" t="s">
-        <v>100</v>
+        <v>133</v>
       </c>
       <c r="B5">
-        <v>3256</v>
+        <v>3232</v>
       </c>
       <c r="C5">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="D5">
-        <v>0.6787575568063373</v>
+        <v>0.6767169179229481</v>
       </c>
       <c r="E5">
-        <v>0.1750614250614251</v>
+        <v>0.1757425742574257</v>
       </c>
       <c r="F5">
-        <v>0.1623931400454414</v>
+        <v>0.1630079693518847</v>
       </c>
       <c r="G5">
-        <v>0.1884955657125316</v>
+        <v>0.1892470977688297</v>
       </c>
       <c r="H5" t="s">
-        <v>101</v>
+        <v>134</v>
       </c>
       <c r="I5" t="s">
-        <v>102</v>
+        <v>135</v>
+      </c>
+      <c r="J5" t="s">
+        <v>136</v>
+      </c>
+      <c r="K5" t="s">
+        <v>137</v>
+      </c>
+      <c r="L5" t="s">
+        <v>138</v>
+      </c>
+      <c r="M5" t="s">
+        <v>139</v>
+      </c>
+      <c r="N5" t="s">
+        <v>140</v>
+      </c>
+      <c r="O5" t="s">
+        <v>141</v>
+      </c>
+      <c r="P5" t="s">
+        <v>142</v>
+      </c>
+      <c r="Q5">
+        <v>0.1757425742574257</v>
       </c>
     </row>
   </sheetData>
@@ -3245,32 +3543,41 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:9">
       <c r="A1" t="s">
-        <v>32</v>
+        <v>57</v>
       </c>
       <c r="B1" t="s">
-        <v>103</v>
+        <v>143</v>
       </c>
       <c r="C1" t="s">
-        <v>104</v>
+        <v>144</v>
       </c>
       <c r="D1" t="s">
-        <v>105</v>
+        <v>145</v>
       </c>
       <c r="E1" t="s">
-        <v>106</v>
+        <v>146</v>
       </c>
       <c r="F1" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6">
+        <v>147</v>
+      </c>
+      <c r="G1" t="s">
+        <v>148</v>
+      </c>
+      <c r="H1" t="s">
+        <v>149</v>
+      </c>
+      <c r="I1" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
       <c r="A2" t="s">
-        <v>108</v>
+        <v>151</v>
       </c>
       <c r="B2">
         <v>26</v>
@@ -3287,70 +3594,106 @@
       <c r="F2">
         <v>26</v>
       </c>
-    </row>
-    <row r="3" spans="1:6">
+      <c r="G2">
+        <v>1</v>
+      </c>
+      <c r="H2">
+        <v>1</v>
+      </c>
+      <c r="I2" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9">
       <c r="A3" t="s">
-        <v>82</v>
+        <v>106</v>
       </c>
       <c r="B3">
-        <v>69.78525641025641</v>
+        <v>62.20857142857143</v>
       </c>
       <c r="C3">
-        <v>33.5</v>
+        <v>27</v>
       </c>
       <c r="D3">
-        <v>624</v>
+        <v>700</v>
       </c>
       <c r="E3">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="F3">
-        <v>81.25</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6">
+        <v>74</v>
+      </c>
+      <c r="G3">
+        <v>740</v>
+      </c>
+      <c r="H3">
+        <v>0.9459459459459459</v>
+      </c>
+      <c r="I3" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9">
       <c r="A4" t="s">
+        <v>103</v>
+      </c>
+      <c r="B4">
+        <v>83.41975308641975</v>
+      </c>
+      <c r="C4">
+        <v>51</v>
+      </c>
+      <c r="D4">
         <v>81</v>
       </c>
-      <c r="B4">
-        <v>93.84722222222223</v>
-      </c>
-      <c r="C4">
-        <v>56.5</v>
-      </c>
-      <c r="D4">
-        <v>72</v>
-      </c>
       <c r="E4">
-        <v>31.75</v>
+        <v>26</v>
       </c>
       <c r="F4">
-        <v>103.25</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6">
+        <v>91</v>
+      </c>
+      <c r="G4">
+        <v>84</v>
+      </c>
+      <c r="H4">
+        <v>0.9642857142857143</v>
+      </c>
+      <c r="I4" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
       <c r="A5" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="B5">
-        <v>86.06779661016949</v>
+        <v>83.7032967032967</v>
       </c>
       <c r="C5">
-        <v>63</v>
+        <v>57.5</v>
       </c>
       <c r="D5">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="E5">
-        <v>28</v>
+        <v>23.5</v>
       </c>
       <c r="F5">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6">
+        <v>100.5</v>
+      </c>
+      <c r="G5">
+        <v>195</v>
+      </c>
+      <c r="H5">
+        <v>0.9333333333333333</v>
+      </c>
+      <c r="I5" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9">
       <c r="A6" t="s">
-        <v>110</v>
+        <v>152</v>
       </c>
       <c r="B6">
         <v>74.41666666666667</v>
@@ -3367,10 +3710,19 @@
       <c r="F6">
         <v>89</v>
       </c>
-    </row>
-    <row r="7" spans="1:6">
+      <c r="G6">
+        <v>24</v>
+      </c>
+      <c r="H6">
+        <v>1</v>
+      </c>
+      <c r="I6" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9">
       <c r="A7" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="B7">
         <v>72.8</v>
@@ -3387,10 +3739,19 @@
       <c r="F7">
         <v>90</v>
       </c>
-    </row>
-    <row r="8" spans="1:6">
+      <c r="G7">
+        <v>5</v>
+      </c>
+      <c r="H7">
+        <v>1</v>
+      </c>
+      <c r="I7" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9">
       <c r="A8" t="s">
-        <v>112</v>
+        <v>153</v>
       </c>
       <c r="B8">
         <v>72</v>
@@ -3407,10 +3768,19 @@
       <c r="F8">
         <v>94.5</v>
       </c>
-    </row>
-    <row r="9" spans="1:6">
+      <c r="G8">
+        <v>2</v>
+      </c>
+      <c r="H8">
+        <v>1</v>
+      </c>
+      <c r="I8" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9">
       <c r="A9" t="s">
-        <v>113</v>
+        <v>154</v>
       </c>
       <c r="B9">
         <v>130.8</v>
@@ -3427,10 +3797,19 @@
       <c r="F9">
         <v>173</v>
       </c>
-    </row>
-    <row r="10" spans="1:6">
+      <c r="G9">
+        <v>5</v>
+      </c>
+      <c r="H9">
+        <v>1</v>
+      </c>
+      <c r="I9" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9">
       <c r="A10" t="s">
-        <v>114</v>
+        <v>104</v>
       </c>
       <c r="B10">
         <v>99.14285714285714</v>
@@ -3447,25 +3826,14 @@
       <c r="F10">
         <v>133.25</v>
       </c>
-    </row>
-    <row r="11" spans="1:6">
-      <c r="A11" t="s">
-        <v>115</v>
-      </c>
-      <c r="B11">
-        <v>262</v>
-      </c>
-      <c r="C11">
-        <v>262</v>
-      </c>
-      <c r="D11">
-        <v>1</v>
-      </c>
-      <c r="E11">
-        <v>262</v>
-      </c>
-      <c r="F11">
-        <v>262</v>
+      <c r="G10">
+        <v>14</v>
+      </c>
+      <c r="H10">
+        <v>1</v>
+      </c>
+      <c r="I10" t="s">
+        <v>155</v>
       </c>
     </row>
   </sheetData>
@@ -3480,18 +3848,18 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" t="s">
-        <v>116</v>
+        <v>156</v>
       </c>
       <c r="B1" t="s">
-        <v>117</v>
+        <v>157</v>
       </c>
       <c r="C1" t="s">
-        <v>118</v>
+        <v>158</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>119</v>
+        <v>159</v>
       </c>
       <c r="B2">
         <v>94</v>
@@ -3502,7 +3870,7 @@
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>120</v>
+        <v>160</v>
       </c>
       <c r="B3">
         <v>18</v>
@@ -3513,7 +3881,7 @@
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>115</v>
+        <v>161</v>
       </c>
       <c r="B4">
         <v>8</v>
@@ -3524,7 +3892,7 @@
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>121</v>
+        <v>162</v>
       </c>
       <c r="B5">
         <v>7</v>
@@ -3545,25 +3913,25 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" t="s">
-        <v>122</v>
+        <v>163</v>
       </c>
       <c r="B1" t="s">
-        <v>117</v>
+        <v>157</v>
       </c>
       <c r="C1" t="s">
-        <v>123</v>
+        <v>164</v>
       </c>
       <c r="D1" t="s">
-        <v>118</v>
+        <v>158</v>
       </c>
       <c r="E1" t="s">
-        <v>124</v>
+        <v>165</v>
       </c>
       <c r="F1" t="s">
-        <v>125</v>
+        <v>166</v>
       </c>
       <c r="G1" t="s">
-        <v>126</v>
+        <v>167</v>
       </c>
     </row>
     <row r="2" spans="1:7">
@@ -3571,22 +3939,22 @@
         <v>0</v>
       </c>
       <c r="B2">
-        <v>2252</v>
+        <v>2245</v>
       </c>
       <c r="C2">
-        <v>825</v>
+        <v>822</v>
       </c>
       <c r="D2">
-        <v>13705715.34</v>
+        <v>13695715.34</v>
       </c>
       <c r="E2">
-        <v>3972380.89</v>
+        <v>3962380.89</v>
       </c>
       <c r="F2">
-        <v>6086.019245115453</v>
+        <v>6100.541354120267</v>
       </c>
       <c r="G2">
-        <v>0.3663410301953819</v>
+        <v>0.3661469933184855</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -3624,110 +3992,110 @@
   <sheetData>
     <row r="1" spans="1:16">
       <c r="A1" t="s">
-        <v>35</v>
+        <v>58</v>
       </c>
       <c r="B1" t="s">
-        <v>127</v>
+        <v>168</v>
       </c>
       <c r="C1" t="s">
-        <v>128</v>
+        <v>169</v>
       </c>
       <c r="D1" t="s">
-        <v>123</v>
+        <v>164</v>
       </c>
       <c r="E1" t="s">
-        <v>118</v>
+        <v>158</v>
       </c>
       <c r="F1" t="s">
-        <v>125</v>
+        <v>166</v>
       </c>
       <c r="G1" t="s">
-        <v>129</v>
+        <v>170</v>
       </c>
       <c r="H1" t="s">
-        <v>130</v>
+        <v>171</v>
       </c>
       <c r="I1" t="s">
-        <v>131</v>
+        <v>172</v>
       </c>
       <c r="J1" t="s">
-        <v>117</v>
+        <v>157</v>
       </c>
       <c r="K1" t="s">
-        <v>126</v>
+        <v>167</v>
       </c>
       <c r="L1" t="s">
-        <v>132</v>
+        <v>173</v>
       </c>
       <c r="M1" t="s">
-        <v>133</v>
+        <v>174</v>
       </c>
       <c r="N1" t="s">
-        <v>134</v>
+        <v>175</v>
       </c>
       <c r="O1" t="s">
-        <v>135</v>
+        <v>176</v>
       </c>
       <c r="P1" t="s">
-        <v>136</v>
+        <v>177</v>
       </c>
     </row>
     <row r="2" spans="1:16">
       <c r="A2" t="s">
-        <v>83</v>
+        <v>108</v>
       </c>
       <c r="B2" t="s">
-        <v>137</v>
+        <v>179</v>
       </c>
       <c r="C2">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="D2">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="E2">
         <v>1723193</v>
       </c>
       <c r="F2">
-        <v>4773.387811634349</v>
+        <v>4786.647222222222</v>
       </c>
       <c r="G2">
         <v>14054</v>
       </c>
       <c r="H2">
-        <v>388</v>
+        <v>383</v>
       </c>
       <c r="I2">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="J2">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="K2">
-        <v>0.5013850415512465</v>
+        <v>0.5</v>
       </c>
       <c r="L2">
-        <v>0.4949561796471565</v>
+        <v>0.4936767143471054</v>
       </c>
       <c r="M2">
-        <v>0.4500639740614632</v>
+        <v>0.4486228630225383</v>
       </c>
       <c r="N2">
-        <v>0.5526769414481715</v>
+        <v>0.5513771369774617</v>
       </c>
       <c r="O2" t="s">
-        <v>140</v>
+        <v>182</v>
       </c>
       <c r="P2">
-        <v>6.956114148761139</v>
+        <v>6.93813254343422</v>
       </c>
     </row>
     <row r="3" spans="1:16">
       <c r="A3" t="s">
-        <v>83</v>
+        <v>108</v>
       </c>
       <c r="B3" t="s">
-        <v>138</v>
+        <v>180</v>
       </c>
       <c r="C3">
         <v>331</v>
@@ -3745,10 +4113,10 @@
         <v>15000</v>
       </c>
       <c r="H3">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="I3">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="J3">
         <v>331</v>
@@ -3757,7 +4125,7 @@
         <v>0.4622356495468278</v>
       </c>
       <c r="L3">
-        <v>0.4585259452688039</v>
+        <v>0.4585427107905017</v>
       </c>
       <c r="M3">
         <v>0.4092643505787315</v>
@@ -3766,18 +4134,18 @@
         <v>0.5160734808018378</v>
       </c>
       <c r="O3" t="s">
-        <v>140</v>
+        <v>182</v>
       </c>
       <c r="P3">
-        <v>6.877889179032058</v>
+        <v>6.878140661857526</v>
       </c>
     </row>
     <row r="4" spans="1:16">
       <c r="A4" t="s">
-        <v>85</v>
+        <v>178</v>
       </c>
       <c r="B4" t="s">
-        <v>137</v>
+        <v>179</v>
       </c>
       <c r="C4">
         <v>6</v>
@@ -3807,7 +4175,7 @@
         <v>0</v>
       </c>
       <c r="L4">
-        <v>0.3479962845010616</v>
+        <v>0.3481644054269752</v>
       </c>
       <c r="M4">
         <v>0</v>
@@ -3816,71 +4184,71 @@
         <v>0.3903430336530645</v>
       </c>
       <c r="O4" t="s">
-        <v>141</v>
+        <v>183</v>
       </c>
       <c r="P4">
-        <v>6.524930334394904</v>
+        <v>6.528082601755786</v>
       </c>
     </row>
     <row r="5" spans="1:16">
       <c r="A5" t="s">
-        <v>83</v>
+        <v>108</v>
       </c>
       <c r="B5" t="s">
-        <v>139</v>
+        <v>181</v>
       </c>
       <c r="C5">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D5">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E5">
         <v>1130483</v>
       </c>
       <c r="F5">
-        <v>7388.777777777777</v>
+        <v>7437.388157894737</v>
       </c>
       <c r="G5">
         <v>15000</v>
       </c>
       <c r="H5">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="I5">
         <v>21</v>
       </c>
       <c r="J5">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="K5">
-        <v>0.4183006535947713</v>
+        <v>0.4144736842105263</v>
       </c>
       <c r="L5">
-        <v>0.4181850614319028</v>
+        <v>0.4150215307437973</v>
       </c>
       <c r="M5">
-        <v>0.3430755238885709</v>
+        <v>0.3392075569039762</v>
       </c>
       <c r="N5">
-        <v>0.4975279894650293</v>
+        <v>0.4939563736511516</v>
       </c>
       <c r="O5" t="s">
-        <v>140</v>
+        <v>182</v>
       </c>
       <c r="P5">
-        <v>6.272775921478542</v>
+        <v>6.22532296115696</v>
       </c>
     </row>
     <row r="6" spans="1:16">
       <c r="A6" t="s">
-        <v>84</v>
+        <v>109</v>
       </c>
       <c r="B6" t="s">
-        <v>139</v>
+        <v>181</v>
       </c>
       <c r="C6">
-        <v>992</v>
+        <v>988</v>
       </c>
       <c r="D6">
         <v>382</v>
@@ -3889,45 +4257,45 @@
         <v>6567606.03</v>
       </c>
       <c r="F6">
-        <v>6620.570594758065</v>
+        <v>6647.374524291498</v>
       </c>
       <c r="G6">
         <v>14000</v>
       </c>
       <c r="H6">
-        <v>1196</v>
+        <v>1177</v>
       </c>
       <c r="I6">
-        <v>204</v>
+        <v>189</v>
       </c>
       <c r="J6">
-        <v>992</v>
+        <v>988</v>
       </c>
       <c r="K6">
-        <v>0.3850806451612903</v>
+        <v>0.3866396761133603</v>
       </c>
       <c r="L6">
-        <v>0.3860350941702918</v>
+        <v>0.3875578768127418</v>
       </c>
       <c r="M6">
-        <v>0.3552971344929201</v>
+        <v>0.3567683527963075</v>
       </c>
       <c r="N6">
-        <v>0.4157507912012866</v>
+        <v>0.417389133641043</v>
       </c>
       <c r="O6" t="s">
-        <v>140</v>
+        <v>182</v>
       </c>
       <c r="P6">
-        <v>5.404491318384085</v>
+        <v>5.425810275378385</v>
       </c>
     </row>
     <row r="7" spans="1:16">
       <c r="A7" t="s">
-        <v>84</v>
+        <v>109</v>
       </c>
       <c r="B7" t="s">
-        <v>137</v>
+        <v>179</v>
       </c>
       <c r="C7">
         <v>23</v>
@@ -3957,7 +4325,7 @@
         <v>0.391304347826087</v>
       </c>
       <c r="L7">
-        <v>0.406186155510155</v>
+        <v>0.4063003508560586</v>
       </c>
       <c r="M7">
         <v>0.2215737798238215</v>
@@ -3966,18 +4334,18 @@
         <v>0.5921482039625402</v>
       </c>
       <c r="O7" t="s">
-        <v>141</v>
+        <v>183</v>
       </c>
       <c r="P7">
-        <v>5.077326943876938</v>
+        <v>5.078754385700733</v>
       </c>
     </row>
     <row r="8" spans="1:16">
       <c r="A8" t="s">
-        <v>84</v>
+        <v>109</v>
       </c>
       <c r="B8" t="s">
-        <v>138</v>
+        <v>180</v>
       </c>
       <c r="C8">
         <v>283</v>
@@ -3995,10 +4363,10 @@
         <v>14170</v>
       </c>
       <c r="H8">
-        <v>350</v>
+        <v>344</v>
       </c>
       <c r="I8">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="J8">
         <v>283</v>
@@ -4007,7 +4375,7 @@
         <v>0.3392226148409894</v>
       </c>
       <c r="L8">
-        <v>0.3467343969394192</v>
+        <v>0.3467537335315371</v>
       </c>
       <c r="M8">
         <v>0.2865431073886124</v>
@@ -4016,18 +4384,18 @@
         <v>0.3962086273667369</v>
       </c>
       <c r="O8" t="s">
-        <v>140</v>
+        <v>182</v>
       </c>
       <c r="P8">
-        <v>4.913226404631571</v>
+        <v>4.913500404141881</v>
       </c>
     </row>
     <row r="9" spans="1:16">
       <c r="A9" t="s">
-        <v>85</v>
+        <v>178</v>
       </c>
       <c r="B9" t="s">
-        <v>138</v>
+        <v>180</v>
       </c>
       <c r="C9">
         <v>215</v>
@@ -4045,10 +4413,10 @@
         <v>10000</v>
       </c>
       <c r="H9">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="I9">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="J9">
         <v>215</v>
@@ -4057,7 +4425,7 @@
         <v>0.4837209302325581</v>
       </c>
       <c r="L9">
-        <v>0.475623943845054</v>
+        <v>0.4756486473280453</v>
       </c>
       <c r="M9">
         <v>0.4177949763281722</v>
@@ -4066,18 +4434,18 @@
         <v>0.5502184178345464</v>
       </c>
       <c r="O9" t="s">
-        <v>140</v>
+        <v>182</v>
       </c>
       <c r="P9">
-        <v>4.75623943845054</v>
+        <v>4.756486473280454</v>
       </c>
     </row>
     <row r="10" spans="1:16">
       <c r="A10" t="s">
-        <v>85</v>
+        <v>178</v>
       </c>
       <c r="B10" t="s">
-        <v>139</v>
+        <v>181</v>
       </c>
       <c r="C10">
         <v>148</v>
@@ -4095,10 +4463,10 @@
         <v>10550</v>
       </c>
       <c r="H10">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="I10">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="J10">
         <v>148</v>
@@ -4107,7 +4475,7 @@
         <v>0.4054054054054054</v>
       </c>
       <c r="L10">
-        <v>0.4074599227080798</v>
+        <v>0.4074939246930961</v>
       </c>
       <c r="M10">
         <v>0.3296683026402324</v>
@@ -4116,10 +4484,10 @@
         <v>0.4859290040267155</v>
       </c>
       <c r="O10" t="s">
-        <v>140</v>
+        <v>182</v>
       </c>
       <c r="P10">
-        <v>4.298702184570242</v>
+        <v>4.299060905512164</v>
       </c>
     </row>
   </sheetData>

</xml_diff>